<commit_message>
modified text file with stellar params
</commit_message>
<xml_diff>
--- a/text_files/combined_yso_parameters_v2.xlsx
+++ b/text_files/combined_yso_parameters_v2.xlsx
@@ -3652,28 +3652,28 @@
     <t xml:space="preserve">OPHIRS63</t>
   </si>
   <si>
-    <t xml:space="preserve">3400.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">200.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">200.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">325.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47.00</t>
+    <t xml:space="preserve">3650.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">300.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.00</t>
   </si>
   <si>
     <t xml:space="preserve">0.309</t>
@@ -4537,7 +4537,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CB35"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.92"/>
@@ -10714,7 +10714,7 @@
         <v>1215</v>
       </c>
       <c r="J29" s="0" t="s">
-        <v>1216</v>
+        <v>550</v>
       </c>
       <c r="K29" s="0" t="s">
         <v>149</v>
@@ -10732,13 +10732,13 @@
         <v>358</v>
       </c>
       <c r="P29" s="0" t="s">
-        <v>401</v>
+        <v>661</v>
       </c>
       <c r="Q29" s="0" t="s">
-        <v>99</v>
+        <v>1216</v>
       </c>
       <c r="R29" s="0" t="s">
-        <v>402</v>
+        <v>98</v>
       </c>
       <c r="S29" s="0" t="s">
         <v>1217</v>
@@ -10747,7 +10747,7 @@
         <v>98</v>
       </c>
       <c r="U29" s="0" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="V29" s="0" t="n">
         <v>0.198</v>

</xml_diff>

<commit_message>
added new protostar classification plots
</commit_message>
<xml_diff>
--- a/text_files/combined_yso_parameters_v2.xlsx
+++ b/text_files/combined_yso_parameters_v2.xlsx
@@ -439,757 +439,757 @@
     <t xml:space="preserve">C18O</t>
   </si>
   <si>
+    <t xml:space="preserve">no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DoAr25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOAR25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3697.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60.89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">351.84</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0231</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2492</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1869</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.0807</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.3475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0796</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0580</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-7.737</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.476</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.627</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1627</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0897</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.567</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-7.348</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.441</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.610</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DoAr43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOAR43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4223.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57.92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">365.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34.57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.565</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.936</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-32.7168</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-35.0692</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-38.1327</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.4275</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.4395</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.2751</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1592</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-15.742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.074</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2629</t>
+  </si>
+  <si>
+    <t xml:space="preserve">127.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.334</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-10.548</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42.449</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.199</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.396</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EC92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3747.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">78.57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">289.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.91</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46.71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5966</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6736</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6611</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6415</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.391</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1822</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.672</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.135</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.914</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.098</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.681</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.135</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2783</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1796</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.637</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.976</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.638</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.892</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.185</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unclear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elia32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIA32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3387.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">279.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.94</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.295</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.859</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2944</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6636</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1296</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.483</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.378</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.856</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.739</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2432</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.765</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.872</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elia33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIA33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3290.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">88.51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87.44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">293.87</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4933</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4397</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4352</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0890</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.548</t>
+  </si>
+  <si>
+    <t xml:space="preserve">62.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.514</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.932</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.538</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2132</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.949</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.446</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.237</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.196</t>
+  </si>
+  <si>
     <t xml:space="preserve">yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DoAr25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOAR25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3697.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60.47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60.89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">351.84</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14.27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.076</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.208</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1642</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0231</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2492</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1869</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.0807</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.3475</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7364</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0796</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0580</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-7.737</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.476</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.627</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.198</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.063</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1627</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0897</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.567</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-7.348</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.441</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.531</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.065</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.610</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DoAr43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOAR43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4223.49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64.13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">57.92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">365.24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13.48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20.03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.95</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34.57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.565</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.936</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-32.7168</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-35.0692</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-38.1327</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.4275</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.4395</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.2751</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.8725</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1592</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.208</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-15.742</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.074</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2629</t>
-  </si>
-  <si>
-    <t xml:space="preserve">127.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.334</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-10.548</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42.449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.199</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.396</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EC92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3747.47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">78.57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">289.04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.91</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">46.71</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6089</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5966</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5817</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6736</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6611</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6415</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.391</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1822</t>
-  </si>
-  <si>
-    <t xml:space="preserve">63.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0837</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.618</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.672</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.135</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.098</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.681</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.135</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2783</t>
-  </si>
-  <si>
-    <t xml:space="preserve">32.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1796</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.637</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.976</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.638</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.892</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.209</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.185</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unclear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elia32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELIA32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3387.46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52.98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">59.98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">279.04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.94</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.295</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.859</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2944</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6162</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.3078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.3034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.6636</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">61.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1296</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.483</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.174</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.378</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.856</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.107</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2432</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.765</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.872</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.795</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.848</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.238</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.228</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elia33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELIA33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3290.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">88.51</t>
-  </si>
-  <si>
-    <t xml:space="preserve">87.44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">293.87</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.68</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.51</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45.45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4933</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7215</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4397</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4352</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.7261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0890</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.548</t>
-  </si>
-  <si>
-    <t xml:space="preserve">62.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.514</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.932</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.538</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.076</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.4252</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2132</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.795</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.949</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.446</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.094</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.237</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.088</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.196</t>
   </si>
   <si>
     <t xml:space="preserve">FP-Tau</t>
@@ -4537,7 +4537,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CB35"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.92"/>
@@ -5232,66 +5232,66 @@
         <v>0.0380628402368316</v>
       </c>
       <c r="CB3" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>193</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>194</v>
       </c>
       <c r="C4" s="0" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="E4" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="F4" s="0" t="s">
         <v>196</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="G4" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="H4" s="0" t="s">
         <v>198</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="I4" s="0" t="s">
         <v>199</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="J4" s="0" t="s">
         <v>200</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="K4" s="0" t="s">
         <v>201</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="L4" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="M4" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="L4" s="0" t="s">
-        <v>202</v>
-      </c>
-      <c r="M4" s="0" t="s">
+      <c r="N4" s="0" t="s">
         <v>203</v>
       </c>
-      <c r="N4" s="0" t="s">
+      <c r="O4" s="0" t="s">
         <v>204</v>
       </c>
-      <c r="O4" s="0" t="s">
+      <c r="P4" s="0" t="s">
         <v>205</v>
       </c>
-      <c r="P4" s="0" t="s">
+      <c r="Q4" s="0" t="s">
         <v>206</v>
       </c>
-      <c r="Q4" s="0" t="s">
+      <c r="R4" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="S4" s="0" t="s">
         <v>207</v>
-      </c>
-      <c r="R4" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="S4" s="0" t="s">
-        <v>208</v>
       </c>
       <c r="T4" s="0" t="s">
         <v>95</v>
@@ -5309,118 +5309,118 @@
         <v>1174.736</v>
       </c>
       <c r="Y4" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="Z4" s="0" t="s">
         <v>209</v>
       </c>
-      <c r="Z4" s="0" t="s">
+      <c r="AA4" s="0" t="s">
         <v>210</v>
-      </c>
-      <c r="AA4" s="0" t="s">
-        <v>211</v>
       </c>
       <c r="AB4" s="0" t="s">
         <v>111</v>
       </c>
       <c r="AC4" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD4" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="AE4" s="0" t="s">
         <v>212</v>
       </c>
-      <c r="AE4" s="0" t="s">
+      <c r="AF4" s="0" t="s">
         <v>213</v>
       </c>
-      <c r="AF4" s="0" t="s">
+      <c r="AG4" s="0" t="s">
         <v>214</v>
       </c>
-      <c r="AG4" s="0" t="s">
+      <c r="AH4" s="0" t="s">
         <v>215</v>
       </c>
-      <c r="AH4" s="0" t="s">
+      <c r="AI4" s="0" t="s">
         <v>216</v>
       </c>
-      <c r="AI4" s="0" t="s">
+      <c r="AJ4" s="0" t="s">
         <v>217</v>
       </c>
-      <c r="AJ4" s="0" t="s">
+      <c r="AK4" s="0" t="s">
         <v>218</v>
       </c>
-      <c r="AK4" s="0" t="s">
+      <c r="AL4" s="0" t="s">
         <v>219</v>
       </c>
-      <c r="AL4" s="0" t="s">
+      <c r="AM4" s="0" t="s">
         <v>220</v>
       </c>
-      <c r="AM4" s="0" t="s">
+      <c r="AN4" s="0" t="s">
         <v>221</v>
       </c>
-      <c r="AN4" s="0" t="s">
+      <c r="AO4" s="0" t="s">
         <v>222</v>
       </c>
-      <c r="AO4" s="0" t="s">
+      <c r="AP4" s="0" t="s">
         <v>223</v>
       </c>
-      <c r="AP4" s="0" t="s">
+      <c r="AQ4" s="0" t="s">
         <v>224</v>
       </c>
-      <c r="AQ4" s="0" t="s">
+      <c r="AR4" s="0" t="s">
         <v>225</v>
       </c>
-      <c r="AR4" s="0" t="s">
+      <c r="AS4" s="0" t="s">
         <v>226</v>
       </c>
-      <c r="AS4" s="0" t="s">
+      <c r="AT4" s="0" t="s">
         <v>227</v>
       </c>
-      <c r="AT4" s="0" t="s">
+      <c r="AU4" s="0" t="s">
         <v>228</v>
       </c>
-      <c r="AU4" s="0" t="s">
+      <c r="AV4" s="0" t="s">
         <v>229</v>
       </c>
-      <c r="AV4" s="0" t="s">
+      <c r="AW4" s="0" t="s">
         <v>230</v>
-      </c>
-      <c r="AW4" s="0" t="s">
-        <v>231</v>
       </c>
       <c r="AX4" s="0" t="s">
         <v>125</v>
       </c>
       <c r="AY4" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="AZ4" s="0" t="s">
         <v>232</v>
-      </c>
-      <c r="AZ4" s="0" t="s">
-        <v>233</v>
       </c>
       <c r="BA4" s="0" t="s">
         <v>111</v>
       </c>
       <c r="BB4" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="BC4" s="0" t="s">
         <v>111</v>
       </c>
       <c r="BD4" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="BE4" s="0" t="s">
         <v>235</v>
       </c>
-      <c r="BE4" s="0" t="s">
+      <c r="BF4" s="0" t="s">
         <v>236</v>
       </c>
-      <c r="BF4" s="0" t="s">
+      <c r="BG4" s="0" t="s">
         <v>237</v>
-      </c>
-      <c r="BG4" s="0" t="s">
-        <v>238</v>
       </c>
       <c r="BH4" s="0" t="s">
         <v>111</v>
       </c>
       <c r="BI4" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="BJ4" s="0" t="s">
         <v>239</v>
-      </c>
-      <c r="BJ4" s="0" t="s">
-        <v>240</v>
       </c>
       <c r="BK4" s="0" t="s">
         <v>138</v>
@@ -5450,72 +5450,72 @@
         <v>0.0101151995020567</v>
       </c>
       <c r="CB4" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C5" s="0" t="n">
         <v>8</v>
       </c>
       <c r="D5" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="E5" s="0" t="s">
         <v>242</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="0" t="s">
         <v>243</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="G5" s="0" t="s">
         <v>244</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="H5" s="0" t="s">
         <v>245</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="I5" s="0" t="s">
         <v>246</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="J5" s="0" t="s">
         <v>247</v>
       </c>
-      <c r="J5" s="0" t="s">
+      <c r="K5" s="0" t="s">
         <v>248</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="L5" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="M5" s="0" t="s">
         <v>249</v>
       </c>
-      <c r="L5" s="0" t="s">
-        <v>249</v>
-      </c>
-      <c r="M5" s="0" t="s">
+      <c r="N5" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="O5" s="0" t="s">
         <v>250</v>
       </c>
-      <c r="N5" s="0" t="s">
-        <v>207</v>
-      </c>
-      <c r="O5" s="0" t="s">
+      <c r="P5" s="0" t="s">
         <v>251</v>
-      </c>
-      <c r="P5" s="0" t="s">
-        <v>252</v>
       </c>
       <c r="Q5" s="0" t="s">
         <v>96</v>
       </c>
       <c r="R5" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="S5" s="0" t="s">
         <v>253</v>
       </c>
-      <c r="S5" s="0" t="s">
+      <c r="T5" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="U5" s="0" t="s">
         <v>254</v>
-      </c>
-      <c r="T5" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="U5" s="0" t="s">
-        <v>255</v>
       </c>
       <c r="V5" s="0" t="n">
         <v>0.688</v>
@@ -5527,118 +5527,118 @@
         <v>508.048</v>
       </c>
       <c r="Y5" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="Z5" s="0" t="s">
         <v>256</v>
       </c>
-      <c r="Z5" s="0" t="s">
+      <c r="AA5" s="0" t="s">
         <v>257</v>
       </c>
-      <c r="AA5" s="0" t="s">
+      <c r="AB5" s="0" t="s">
         <v>258</v>
       </c>
-      <c r="AB5" s="0" t="s">
+      <c r="AC5" s="0" t="s">
         <v>259</v>
       </c>
-      <c r="AC5" s="0" t="s">
+      <c r="AD5" s="0" t="s">
         <v>260</v>
       </c>
-      <c r="AD5" s="0" t="s">
+      <c r="AE5" s="0" t="s">
         <v>261</v>
       </c>
-      <c r="AE5" s="0" t="s">
+      <c r="AF5" s="0" t="s">
         <v>262</v>
       </c>
-      <c r="AF5" s="0" t="s">
+      <c r="AG5" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="AG5" s="0" t="s">
+      <c r="AH5" s="0" t="s">
         <v>264</v>
       </c>
-      <c r="AH5" s="0" t="s">
+      <c r="AI5" s="0" t="s">
         <v>265</v>
       </c>
-      <c r="AI5" s="0" t="s">
+      <c r="AJ5" s="0" t="s">
         <v>266</v>
       </c>
-      <c r="AJ5" s="0" t="s">
+      <c r="AK5" s="0" t="s">
         <v>267</v>
       </c>
-      <c r="AK5" s="0" t="s">
+      <c r="AL5" s="0" t="s">
         <v>268</v>
       </c>
-      <c r="AL5" s="0" t="s">
+      <c r="AM5" s="0" t="s">
         <v>269</v>
       </c>
-      <c r="AM5" s="0" t="s">
+      <c r="AN5" s="0" t="s">
         <v>270</v>
       </c>
-      <c r="AN5" s="0" t="s">
+      <c r="AO5" s="0" t="s">
         <v>271</v>
       </c>
-      <c r="AO5" s="0" t="s">
+      <c r="AP5" s="0" t="s">
         <v>272</v>
       </c>
-      <c r="AP5" s="0" t="s">
+      <c r="AQ5" s="0" t="s">
         <v>273</v>
       </c>
-      <c r="AQ5" s="0" t="s">
+      <c r="AR5" s="0" t="s">
         <v>274</v>
       </c>
-      <c r="AR5" s="0" t="s">
+      <c r="AS5" s="0" t="s">
         <v>275</v>
       </c>
-      <c r="AS5" s="0" t="s">
+      <c r="AT5" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="AT5" s="0" t="s">
+      <c r="AU5" s="0" t="s">
         <v>277</v>
       </c>
-      <c r="AU5" s="0" t="s">
+      <c r="AV5" s="0" t="s">
         <v>278</v>
       </c>
-      <c r="AV5" s="0" t="s">
+      <c r="AW5" s="0" t="s">
         <v>279</v>
-      </c>
-      <c r="AW5" s="0" t="s">
-        <v>280</v>
       </c>
       <c r="AX5" s="0" t="s">
         <v>125</v>
       </c>
       <c r="AY5" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="AZ5" s="0" t="s">
         <v>281</v>
       </c>
-      <c r="AZ5" s="0" t="s">
+      <c r="BA5" s="0" t="s">
         <v>282</v>
       </c>
-      <c r="BA5" s="0" t="s">
+      <c r="BB5" s="0" t="s">
         <v>283</v>
       </c>
-      <c r="BB5" s="0" t="s">
+      <c r="BC5" s="0" t="s">
         <v>284</v>
       </c>
-      <c r="BC5" s="0" t="s">
+      <c r="BD5" s="0" t="s">
         <v>285</v>
       </c>
-      <c r="BD5" s="0" t="s">
+      <c r="BE5" s="0" t="s">
         <v>286</v>
       </c>
-      <c r="BE5" s="0" t="s">
+      <c r="BF5" s="0" t="s">
         <v>287</v>
       </c>
-      <c r="BF5" s="0" t="s">
+      <c r="BG5" s="0" t="s">
         <v>288</v>
       </c>
-      <c r="BG5" s="0" t="s">
+      <c r="BH5" s="0" t="s">
         <v>289</v>
       </c>
-      <c r="BH5" s="0" t="s">
+      <c r="BI5" s="0" t="s">
         <v>290</v>
       </c>
-      <c r="BI5" s="0" t="s">
+      <c r="BJ5" s="0" t="s">
         <v>291</v>
-      </c>
-      <c r="BJ5" s="0" t="s">
-        <v>292</v>
       </c>
       <c r="BK5" s="0" t="s">
         <v>138</v>
@@ -5668,72 +5668,72 @@
         <v>0.666421707762511</v>
       </c>
       <c r="CB5" s="0" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>294</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>295</v>
       </c>
       <c r="C6" s="0" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="0" t="s">
+        <v>295</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>296</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="F6" s="0" t="s">
         <v>297</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>298</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="H6" s="0" t="s">
         <v>299</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="I6" s="0" t="s">
         <v>300</v>
-      </c>
-      <c r="I6" s="0" t="s">
-        <v>301</v>
       </c>
       <c r="J6" s="0" t="s">
         <v>151</v>
       </c>
       <c r="K6" s="0" t="s">
+        <v>301</v>
+      </c>
+      <c r="L6" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="M6" s="0" t="s">
         <v>302</v>
       </c>
-      <c r="L6" s="0" t="s">
-        <v>258</v>
-      </c>
-      <c r="M6" s="0" t="s">
+      <c r="N6" s="0" t="s">
         <v>303</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="O6" s="0" t="s">
         <v>304</v>
       </c>
-      <c r="O6" s="0" t="s">
+      <c r="P6" s="0" t="s">
         <v>305</v>
       </c>
-      <c r="P6" s="0" t="s">
+      <c r="Q6" s="0" t="s">
         <v>306</v>
       </c>
-      <c r="Q6" s="0" t="s">
+      <c r="R6" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="S6" s="0" t="s">
         <v>307</v>
       </c>
-      <c r="R6" s="0" t="s">
-        <v>202</v>
-      </c>
-      <c r="S6" s="0" t="s">
-        <v>308</v>
-      </c>
       <c r="T6" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="U6" s="0" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="V6" s="0" t="n">
         <v>-0.263</v>
@@ -5745,118 +5745,118 @@
         <v>95.74</v>
       </c>
       <c r="Y6" s="0" t="s">
+        <v>308</v>
+      </c>
+      <c r="Z6" s="0" t="s">
         <v>309</v>
       </c>
-      <c r="Z6" s="0" t="s">
+      <c r="AA6" s="0" t="s">
         <v>310</v>
       </c>
-      <c r="AA6" s="0" t="s">
+      <c r="AB6" s="0" t="s">
         <v>311</v>
       </c>
-      <c r="AB6" s="0" t="s">
+      <c r="AC6" s="0" t="s">
         <v>312</v>
       </c>
-      <c r="AC6" s="0" t="s">
+      <c r="AD6" s="0" t="s">
         <v>313</v>
       </c>
-      <c r="AD6" s="0" t="s">
+      <c r="AE6" s="0" t="s">
+        <v>313</v>
+      </c>
+      <c r="AF6" s="0" t="s">
+        <v>313</v>
+      </c>
+      <c r="AG6" s="0" t="s">
         <v>314</v>
       </c>
-      <c r="AE6" s="0" t="s">
-        <v>314</v>
-      </c>
-      <c r="AF6" s="0" t="s">
-        <v>314</v>
-      </c>
-      <c r="AG6" s="0" t="s">
+      <c r="AH6" s="0" t="s">
         <v>315</v>
       </c>
-      <c r="AH6" s="0" t="s">
+      <c r="AI6" s="0" t="s">
         <v>316</v>
       </c>
-      <c r="AI6" s="0" t="s">
+      <c r="AJ6" s="0" t="s">
         <v>317</v>
       </c>
-      <c r="AJ6" s="0" t="s">
+      <c r="AK6" s="0" t="s">
         <v>318</v>
       </c>
-      <c r="AK6" s="0" t="s">
+      <c r="AL6" s="0" t="s">
         <v>319</v>
       </c>
-      <c r="AL6" s="0" t="s">
+      <c r="AM6" s="0" t="s">
         <v>320</v>
       </c>
-      <c r="AM6" s="0" t="s">
+      <c r="AN6" s="0" t="s">
         <v>321</v>
       </c>
-      <c r="AN6" s="0" t="s">
+      <c r="AO6" s="0" t="s">
         <v>322</v>
       </c>
-      <c r="AO6" s="0" t="s">
+      <c r="AP6" s="0" t="s">
         <v>323</v>
       </c>
-      <c r="AP6" s="0" t="s">
+      <c r="AQ6" s="0" t="s">
         <v>324</v>
       </c>
-      <c r="AQ6" s="0" t="s">
+      <c r="AR6" s="0" t="s">
         <v>325</v>
       </c>
-      <c r="AR6" s="0" t="s">
+      <c r="AS6" s="0" t="s">
         <v>326</v>
       </c>
-      <c r="AS6" s="0" t="s">
+      <c r="AT6" s="0" t="s">
         <v>327</v>
       </c>
-      <c r="AT6" s="0" t="s">
+      <c r="AU6" s="0" t="s">
         <v>328</v>
       </c>
-      <c r="AU6" s="0" t="s">
+      <c r="AV6" s="0" t="s">
         <v>329</v>
       </c>
-      <c r="AV6" s="0" t="s">
+      <c r="AW6" s="0" t="s">
         <v>330</v>
-      </c>
-      <c r="AW6" s="0" t="s">
-        <v>331</v>
       </c>
       <c r="AX6" s="0" t="s">
         <v>125</v>
       </c>
       <c r="AY6" s="0" t="s">
+        <v>331</v>
+      </c>
+      <c r="AZ6" s="0" t="s">
         <v>332</v>
       </c>
-      <c r="AZ6" s="0" t="s">
+      <c r="BA6" s="0" t="s">
         <v>333</v>
       </c>
-      <c r="BA6" s="0" t="s">
+      <c r="BB6" s="0" t="s">
         <v>334</v>
       </c>
-      <c r="BB6" s="0" t="s">
+      <c r="BC6" s="0" t="s">
         <v>335</v>
       </c>
-      <c r="BC6" s="0" t="s">
+      <c r="BD6" s="0" t="s">
         <v>336</v>
       </c>
-      <c r="BD6" s="0" t="s">
+      <c r="BE6" s="0" t="s">
         <v>337</v>
       </c>
-      <c r="BE6" s="0" t="s">
+      <c r="BF6" s="0" t="s">
         <v>338</v>
       </c>
-      <c r="BF6" s="0" t="s">
+      <c r="BG6" s="0" t="s">
         <v>339</v>
       </c>
-      <c r="BG6" s="0" t="s">
+      <c r="BH6" s="0" t="s">
         <v>340</v>
       </c>
-      <c r="BH6" s="0" t="s">
+      <c r="BI6" s="0" t="s">
         <v>341</v>
       </c>
-      <c r="BI6" s="0" t="s">
+      <c r="BJ6" s="0" t="s">
         <v>342</v>
-      </c>
-      <c r="BJ6" s="0" t="s">
-        <v>343</v>
       </c>
       <c r="BK6" s="0" t="s">
         <v>138</v>
@@ -5886,72 +5886,72 @@
         <v>0.503607137794084</v>
       </c>
       <c r="CB6" s="0" t="s">
-        <v>139</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>343</v>
+      </c>
+      <c r="B7" s="0" t="s">
         <v>344</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>345</v>
       </c>
       <c r="C7" s="0" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>346</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="F7" s="0" t="s">
         <v>347</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="G7" s="0" t="s">
         <v>348</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="H7" s="0" t="s">
         <v>349</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="I7" s="0" t="s">
         <v>350</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="J7" s="0" t="s">
         <v>351</v>
-      </c>
-      <c r="J7" s="0" t="s">
-        <v>352</v>
       </c>
       <c r="K7" s="0" t="s">
         <v>156</v>
       </c>
       <c r="L7" s="0" t="s">
+        <v>352</v>
+      </c>
+      <c r="M7" s="0" t="s">
         <v>353</v>
       </c>
-      <c r="M7" s="0" t="s">
+      <c r="N7" s="0" t="s">
         <v>354</v>
       </c>
-      <c r="N7" s="0" t="s">
+      <c r="O7" s="0" t="s">
         <v>355</v>
       </c>
-      <c r="O7" s="0" t="s">
+      <c r="P7" s="0" t="s">
         <v>356</v>
       </c>
-      <c r="P7" s="0" t="s">
+      <c r="Q7" s="0" t="s">
+        <v>303</v>
+      </c>
+      <c r="R7" s="0" t="s">
         <v>357</v>
       </c>
-      <c r="Q7" s="0" t="s">
-        <v>304</v>
-      </c>
-      <c r="R7" s="0" t="s">
+      <c r="S7" s="0" t="s">
         <v>358</v>
-      </c>
-      <c r="S7" s="0" t="s">
-        <v>359</v>
       </c>
       <c r="T7" s="0" t="s">
         <v>98</v>
       </c>
       <c r="U7" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="V7" s="0" t="n">
         <v>-0.373</v>
@@ -5963,118 +5963,118 @@
         <v>535.206</v>
       </c>
       <c r="Y7" s="0" t="s">
+        <v>359</v>
+      </c>
+      <c r="Z7" s="0" t="s">
+        <v>309</v>
+      </c>
+      <c r="AA7" s="0" t="s">
         <v>360</v>
       </c>
-      <c r="Z7" s="0" t="s">
-        <v>310</v>
-      </c>
-      <c r="AA7" s="0" t="s">
+      <c r="AB7" s="0" t="s">
         <v>361</v>
       </c>
-      <c r="AB7" s="0" t="s">
+      <c r="AC7" s="0" t="s">
         <v>362</v>
       </c>
-      <c r="AC7" s="0" t="s">
+      <c r="AD7" s="0" t="s">
         <v>363</v>
       </c>
-      <c r="AD7" s="0" t="s">
+      <c r="AE7" s="0" t="s">
+        <v>363</v>
+      </c>
+      <c r="AF7" s="0" t="s">
+        <v>363</v>
+      </c>
+      <c r="AG7" s="0" t="s">
         <v>364</v>
       </c>
-      <c r="AE7" s="0" t="s">
-        <v>364</v>
-      </c>
-      <c r="AF7" s="0" t="s">
-        <v>364</v>
-      </c>
-      <c r="AG7" s="0" t="s">
+      <c r="AH7" s="0" t="s">
         <v>365</v>
       </c>
-      <c r="AH7" s="0" t="s">
+      <c r="AI7" s="0" t="s">
         <v>366</v>
       </c>
-      <c r="AI7" s="0" t="s">
+      <c r="AJ7" s="0" t="s">
         <v>367</v>
       </c>
-      <c r="AJ7" s="0" t="s">
+      <c r="AK7" s="0" t="s">
         <v>368</v>
       </c>
-      <c r="AK7" s="0" t="s">
+      <c r="AL7" s="0" t="s">
+        <v>319</v>
+      </c>
+      <c r="AM7" s="0" t="s">
+        <v>320</v>
+      </c>
+      <c r="AN7" s="0" t="s">
         <v>369</v>
       </c>
-      <c r="AL7" s="0" t="s">
-        <v>320</v>
-      </c>
-      <c r="AM7" s="0" t="s">
-        <v>321</v>
-      </c>
-      <c r="AN7" s="0" t="s">
+      <c r="AO7" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="AO7" s="0" t="s">
+      <c r="AP7" s="0" t="s">
         <v>371</v>
       </c>
-      <c r="AP7" s="0" t="s">
+      <c r="AQ7" s="0" t="s">
         <v>372</v>
       </c>
-      <c r="AQ7" s="0" t="s">
+      <c r="AR7" s="0" t="s">
         <v>373</v>
       </c>
-      <c r="AR7" s="0" t="s">
+      <c r="AS7" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="AT7" s="0" t="s">
         <v>374</v>
       </c>
-      <c r="AS7" s="0" t="s">
-        <v>239</v>
-      </c>
-      <c r="AT7" s="0" t="s">
+      <c r="AU7" s="0" t="s">
         <v>375</v>
       </c>
-      <c r="AU7" s="0" t="s">
+      <c r="AV7" s="0" t="s">
+        <v>329</v>
+      </c>
+      <c r="AW7" s="0" t="s">
         <v>376</v>
-      </c>
-      <c r="AV7" s="0" t="s">
-        <v>330</v>
-      </c>
-      <c r="AW7" s="0" t="s">
-        <v>377</v>
       </c>
       <c r="AX7" s="0" t="s">
         <v>125</v>
       </c>
       <c r="AY7" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="AZ7" s="0" t="s">
         <v>378</v>
       </c>
-      <c r="AZ7" s="0" t="s">
+      <c r="BA7" s="0" t="s">
         <v>379</v>
       </c>
-      <c r="BA7" s="0" t="s">
+      <c r="BB7" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="BB7" s="0" t="s">
+      <c r="BC7" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="BC7" s="0" t="s">
+      <c r="BD7" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="BD7" s="0" t="s">
+      <c r="BE7" s="0" t="s">
         <v>383</v>
       </c>
-      <c r="BE7" s="0" t="s">
+      <c r="BF7" s="0" t="s">
         <v>384</v>
       </c>
-      <c r="BF7" s="0" t="s">
+      <c r="BG7" s="0" t="s">
         <v>385</v>
       </c>
-      <c r="BG7" s="0" t="s">
+      <c r="BH7" s="0" t="s">
         <v>386</v>
       </c>
-      <c r="BH7" s="0" t="s">
+      <c r="BI7" s="0" t="s">
         <v>387</v>
       </c>
-      <c r="BI7" s="0" t="s">
+      <c r="BJ7" s="0" t="s">
         <v>388</v>
-      </c>
-      <c r="BJ7" s="0" t="s">
-        <v>389</v>
       </c>
       <c r="BK7" s="0" t="s">
         <v>138</v>
@@ -6104,7 +6104,7 @@
         <v>0.395803352814387</v>
       </c>
       <c r="CB7" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6151,7 +6151,7 @@
         <v>400</v>
       </c>
       <c r="O8" s="0" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="P8" s="0" t="s">
         <v>401</v>
@@ -6268,7 +6268,7 @@
         <v>417</v>
       </c>
       <c r="BB8" s="0" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="BC8" s="0" t="s">
         <v>418</v>
@@ -6322,7 +6322,7 @@
         <v>0.0090186487762727</v>
       </c>
       <c r="CB8" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6357,16 +6357,16 @@
         <v>434</v>
       </c>
       <c r="K9" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="L9" s="0" t="s">
         <v>202</v>
-      </c>
-      <c r="L9" s="0" t="s">
-        <v>203</v>
       </c>
       <c r="M9" s="0" t="s">
         <v>435</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="O9" s="0" t="s">
         <v>436</v>
@@ -6378,16 +6378,16 @@
         <v>437</v>
       </c>
       <c r="R9" s="0" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="S9" s="0" t="s">
         <v>438</v>
       </c>
       <c r="T9" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="U9" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="V9" s="0" t="n">
         <v>0.912</v>
@@ -6405,7 +6405,7 @@
         <v>440</v>
       </c>
       <c r="AA9" s="0" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="AB9" s="0" t="s">
         <v>441</v>
@@ -6540,7 +6540,7 @@
         <v>0.167673724551042</v>
       </c>
       <c r="CB9" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6575,13 +6575,13 @@
         <v>481</v>
       </c>
       <c r="K10" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L10" s="0" t="s">
         <v>482</v>
       </c>
       <c r="M10" s="0" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="N10" s="0" t="s">
         <v>483</v>
@@ -6620,7 +6620,7 @@
         <v>490</v>
       </c>
       <c r="Z10" s="0" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AA10" s="0" t="s">
         <v>491</v>
@@ -6758,7 +6758,7 @@
         <v>0.16832001551939</v>
       </c>
       <c r="CB10" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6805,13 +6805,13 @@
         <v>534</v>
       </c>
       <c r="O11" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P11" s="0" t="s">
         <v>535</v>
       </c>
       <c r="Q11" s="0" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R11" s="0" t="s">
         <v>156</v>
@@ -6823,7 +6823,7 @@
         <v>537</v>
       </c>
       <c r="U11" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="V11" s="0" t="n">
         <v>-0.727</v>
@@ -6976,7 +6976,7 @@
         <v>0.013289425287221</v>
       </c>
       <c r="CB11" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7011,10 +7011,10 @@
         <v>565</v>
       </c>
       <c r="K12" s="0" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="L12" s="0" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="M12" s="0" t="s">
         <v>566</v>
@@ -7194,7 +7194,7 @@
         <v>0.0029903427221598</v>
       </c>
       <c r="CB12" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7247,7 +7247,7 @@
         <v>608</v>
       </c>
       <c r="Q13" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R13" s="0" t="s">
         <v>609</v>
@@ -7319,7 +7319,7 @@
         <v>617</v>
       </c>
       <c r="AO13" s="0" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AP13" s="0" t="s">
         <v>618</v>
@@ -7379,7 +7379,7 @@
         <v>633</v>
       </c>
       <c r="BI13" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="BJ13" s="0" t="s">
         <v>634</v>
@@ -7412,7 +7412,7 @@
         <v>0.0115888097756542</v>
       </c>
       <c r="CB13" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7465,7 +7465,7 @@
         <v>646</v>
       </c>
       <c r="Q14" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="R14" s="0" t="s">
         <v>486</v>
@@ -7474,10 +7474,10 @@
         <v>647</v>
       </c>
       <c r="T14" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U14" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="V14" s="0" t="n">
         <v>-0.008</v>
@@ -7600,7 +7600,7 @@
         <v>674</v>
       </c>
       <c r="BJ14" s="0" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="BK14" s="0" t="s">
         <v>138</v>
@@ -7630,7 +7630,7 @@
         <v>0.0023432997084543</v>
       </c>
       <c r="CB14" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7662,13 +7662,13 @@
         <v>682</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K15" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M15" s="0" t="s">
         <v>683</v>
@@ -7686,7 +7686,7 @@
         <v>686</v>
       </c>
       <c r="R15" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="S15" s="0" t="s">
         <v>687</v>
@@ -7725,7 +7725,7 @@
         <v>128</v>
       </c>
       <c r="AE15" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AF15" s="0" t="s">
         <v>691</v>
@@ -7794,7 +7794,7 @@
         <v>711</v>
       </c>
       <c r="BB15" s="0" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="BC15" s="0" t="s">
         <v>712</v>
@@ -7848,7 +7848,7 @@
         <v>0.392855759479319</v>
       </c>
       <c r="CB15" s="0" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7883,7 +7883,7 @@
         <v>728</v>
       </c>
       <c r="K16" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L16" s="0" t="s">
         <v>729</v>
@@ -7901,7 +7901,7 @@
         <v>733</v>
       </c>
       <c r="Q16" s="0" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R16" s="0" t="s">
         <v>154</v>
@@ -7910,10 +7910,10 @@
         <v>734</v>
       </c>
       <c r="T16" s="0" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="U16" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="V16" s="0" t="n">
         <v>0.26</v>
@@ -8033,7 +8033,7 @@
         <v>124</v>
       </c>
       <c r="BI16" s="0" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="BJ16" s="0" t="s">
         <v>764</v>
@@ -8066,7 +8066,7 @@
         <v>0.0532175041003053</v>
       </c>
       <c r="CB16" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8101,10 +8101,10 @@
         <v>436</v>
       </c>
       <c r="K17" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M17" s="0" t="s">
         <v>773</v>
@@ -8128,7 +8128,7 @@
         <v>777</v>
       </c>
       <c r="T17" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="U17" s="0" t="s">
         <v>486</v>
@@ -8200,7 +8200,7 @@
         <v>789</v>
       </c>
       <c r="AR17" s="0" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="AS17" s="0" t="s">
         <v>187</v>
@@ -8284,7 +8284,7 @@
         <v>0.0202084420228833</v>
       </c>
       <c r="CB17" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8337,7 +8337,7 @@
         <v>813</v>
       </c>
       <c r="Q18" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="R18" s="0" t="s">
         <v>154</v>
@@ -8346,7 +8346,7 @@
         <v>814</v>
       </c>
       <c r="T18" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="U18" s="0" t="s">
         <v>729</v>
@@ -8427,7 +8427,7 @@
         <v>834</v>
       </c>
       <c r="AU18" s="0" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AV18" s="0" t="s">
         <v>423</v>
@@ -8472,7 +8472,7 @@
         <v>845</v>
       </c>
       <c r="BJ18" s="0" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="BK18" s="0" t="s">
         <v>138</v>
@@ -8546,13 +8546,13 @@
         <v>854</v>
       </c>
       <c r="N19" s="0" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O19" s="0" t="s">
         <v>778</v>
       </c>
       <c r="P19" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Q19" s="0" t="s">
         <v>686</v>
@@ -8720,7 +8720,7 @@
         <v>0.0548659111026197</v>
       </c>
       <c r="CB19" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8755,10 +8755,10 @@
         <v>896</v>
       </c>
       <c r="K20" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L20" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="M20" s="0" t="s">
         <v>897</v>
@@ -8782,7 +8782,7 @@
         <v>899</v>
       </c>
       <c r="T20" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="U20" s="0" t="s">
         <v>151</v>
@@ -8878,7 +8878,7 @@
         <v>922</v>
       </c>
       <c r="AZ20" s="0" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BA20" s="0" t="s">
         <v>923</v>
@@ -8938,7 +8938,7 @@
         <v>0.062955826049373</v>
       </c>
       <c r="CB20" s="0" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8976,7 +8976,7 @@
         <v>482</v>
       </c>
       <c r="L21" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M21" s="0" t="s">
         <v>940</v>
@@ -9066,7 +9066,7 @@
         <v>921</v>
       </c>
       <c r="AP21" s="0" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AQ21" s="0" t="s">
         <v>953</v>
@@ -9156,7 +9156,7 @@
         <v>0.0252706847963137</v>
       </c>
       <c r="CB21" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9194,7 +9194,7 @@
         <v>156</v>
       </c>
       <c r="L22" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="M22" s="0" t="s">
         <v>973</v>
@@ -9209,7 +9209,7 @@
         <v>974</v>
       </c>
       <c r="Q22" s="0" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="R22" s="0" t="s">
         <v>96</v>
@@ -9221,7 +9221,7 @@
         <v>402</v>
       </c>
       <c r="U22" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="V22" s="0" t="n">
         <v>0.145</v>
@@ -9374,7 +9374,7 @@
         <v>0.00527016212505</v>
       </c>
       <c r="CB22" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9409,7 +9409,7 @@
         <v>774</v>
       </c>
       <c r="K23" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="L23" s="0" t="s">
         <v>537</v>
@@ -9421,7 +9421,7 @@
         <v>90</v>
       </c>
       <c r="O23" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="P23" s="0" t="s">
         <v>1008</v>
@@ -9439,7 +9439,7 @@
         <v>732</v>
       </c>
       <c r="U23" s="0" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="V23" s="0" t="n">
         <v>0.535</v>
@@ -9541,7 +9541,7 @@
         <v>1033</v>
       </c>
       <c r="BC23" s="0" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="BD23" s="0" t="s">
         <v>1034</v>
@@ -9592,7 +9592,7 @@
         <v>0.0765617295709479</v>
       </c>
       <c r="CB23" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9627,10 +9627,10 @@
         <v>1048</v>
       </c>
       <c r="K24" s="0" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="L24" s="0" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M24" s="0" t="s">
         <v>1049</v>
@@ -9639,7 +9639,7 @@
         <v>643</v>
       </c>
       <c r="O24" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P24" s="0" t="s">
         <v>1050</v>
@@ -9774,7 +9774,7 @@
         <v>1081</v>
       </c>
       <c r="BH24" s="0" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="BI24" s="0" t="s">
         <v>1082</v>
@@ -9810,7 +9810,7 @@
         <v>0.0081524914819445</v>
       </c>
       <c r="CB24" s="0" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9869,7 +9869,7 @@
         <v>1096</v>
       </c>
       <c r="S25" s="0" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="T25" s="0" t="s">
         <v>1097</v>
@@ -9977,7 +9977,7 @@
         <v>1118</v>
       </c>
       <c r="BC25" s="0" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="BD25" s="0" t="s">
         <v>1119</v>
@@ -10028,7 +10028,7 @@
         <v>0.0235870262330728</v>
       </c>
       <c r="CB25" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10060,28 +10060,28 @@
         <v>1129</v>
       </c>
       <c r="J26" s="0" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K26" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L26" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M26" s="0" t="s">
         <v>98</v>
       </c>
       <c r="N26" s="0" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="O26" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="P26" s="0" t="s">
         <v>1130</v>
       </c>
       <c r="Q26" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R26" s="0" t="s">
         <v>98</v>
@@ -10216,7 +10216,7 @@
         <v>919</v>
       </c>
       <c r="BJ26" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="BK26" s="0" t="s">
         <v>138</v>
@@ -10246,7 +10246,7 @@
         <v>0.0106133151778276</v>
       </c>
       <c r="CB26" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10281,10 +10281,10 @@
         <v>773</v>
       </c>
       <c r="K27" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L27" s="0" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M27" s="0" t="s">
         <v>489</v>
@@ -10293,7 +10293,7 @@
         <v>1161</v>
       </c>
       <c r="O27" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="P27" s="0" t="s">
         <v>1162</v>
@@ -10434,7 +10434,7 @@
         <v>919</v>
       </c>
       <c r="BJ27" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="BK27" s="0" t="s">
         <v>138</v>
@@ -10464,7 +10464,7 @@
         <v>0.0106133151778276</v>
       </c>
       <c r="CB27" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10499,7 +10499,7 @@
         <v>90</v>
       </c>
       <c r="K28" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L28" s="0" t="s">
         <v>1171</v>
@@ -10682,7 +10682,7 @@
         <v>0.743573795357449</v>
       </c>
       <c r="CB28" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10729,7 +10729,7 @@
         <v>400</v>
       </c>
       <c r="O29" s="0" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="P29" s="0" t="s">
         <v>661</v>
@@ -10762,7 +10762,7 @@
         <v>1218</v>
       </c>
       <c r="Z29" s="0" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AA29" s="0" t="s">
         <v>1219</v>
@@ -10828,7 +10828,7 @@
         <v>137</v>
       </c>
       <c r="AV29" s="0" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AW29" s="0" t="s">
         <v>1239</v>
@@ -10900,7 +10900,7 @@
         <v>0.0991567793048796</v>
       </c>
       <c r="CB29" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11118,7 +11118,7 @@
         <v>0.0131063361209077</v>
       </c>
       <c r="CB30" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11159,10 +11159,10 @@
         <v>1171</v>
       </c>
       <c r="M31" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="N31" s="0" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="O31" s="0" t="s">
         <v>154</v>
@@ -11171,7 +11171,7 @@
         <v>1294</v>
       </c>
       <c r="Q31" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="R31" s="0" t="s">
         <v>1171</v>
@@ -11336,7 +11336,7 @@
         <v>0.261757180174782</v>
       </c>
       <c r="CB31" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11371,10 +11371,10 @@
         <v>1331</v>
       </c>
       <c r="K32" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L32" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="M32" s="0" t="s">
         <v>1098</v>
@@ -11389,10 +11389,10 @@
         <v>1332</v>
       </c>
       <c r="Q32" s="0" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R32" s="0" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="S32" s="0" t="s">
         <v>1333</v>
@@ -11401,7 +11401,7 @@
         <v>156</v>
       </c>
       <c r="U32" s="0" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="V32" s="0" t="n">
         <v>-0.217</v>
@@ -11464,7 +11464,7 @@
         <v>1340</v>
       </c>
       <c r="AP32" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="AQ32" s="0" t="s">
         <v>1341</v>
@@ -11524,7 +11524,7 @@
         <v>1352</v>
       </c>
       <c r="BJ32" s="0" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="BK32" s="0" t="s">
         <v>138</v>
@@ -11554,7 +11554,7 @@
         <v>0.0066831881076731</v>
       </c>
       <c r="CB32" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11592,7 +11592,7 @@
         <v>537</v>
       </c>
       <c r="L33" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M33" s="0" t="s">
         <v>1259</v>
@@ -11691,7 +11691,7 @@
         <v>1377</v>
       </c>
       <c r="AS33" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AT33" s="0" t="s">
         <v>1179</v>
@@ -11772,7 +11772,7 @@
         <v>0.0203824306962105</v>
       </c>
       <c r="CB33" s="0" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11804,7 +11804,7 @@
         <v>836</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K34" s="0" t="s">
         <v>398</v>
@@ -11825,7 +11825,7 @@
         <v>1393</v>
       </c>
       <c r="Q34" s="0" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R34" s="0" t="s">
         <v>154</v>
@@ -11852,7 +11852,7 @@
         <v>124</v>
       </c>
       <c r="Z34" s="0" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AA34" s="0" t="s">
         <v>1395</v>
@@ -11909,7 +11909,7 @@
         <v>1410</v>
       </c>
       <c r="AS34" s="0" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AT34" s="0" t="s">
         <v>1411</v>
@@ -11960,7 +11960,7 @@
         <v>1422</v>
       </c>
       <c r="BJ34" s="0" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="BK34" s="0" t="s">
         <v>138</v>
@@ -11990,7 +11990,7 @@
         <v>0.353649091064213</v>
       </c>
       <c r="CB34" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12028,7 +12028,7 @@
         <v>154</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M35" s="0" t="s">
         <v>1431</v>
@@ -12043,7 +12043,7 @@
         <v>608</v>
       </c>
       <c r="Q35" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R35" s="0" t="s">
         <v>482</v>
@@ -12052,10 +12052,10 @@
         <v>1432</v>
       </c>
       <c r="T35" s="0" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="U35" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="V35" s="0" t="n">
         <v>-0.751</v>
@@ -12208,7 +12208,7 @@
         <v>0.130179253064501</v>
       </c>
       <c r="CB35" s="0" t="s">
-        <v>192</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>